<commit_message>
Fix #NAME? on XLOOKUP: it needs the _xlfn. prefix like FORMULATEXT
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0165WQeoaB3CPsnpvD7o3Yah
</commit_message>
<xml_diff>
--- a/textbook_examples/mod01_lookup.xlsx
+++ b/textbook_examples/mod01_lookup.xlsx
@@ -580,7 +580,7 @@
         <v>41.2</v>
       </c>
       <c r="E5" s="9">
-        <f>XLOOKUP(B5,$H$5:$H$7,$I$5:$I$7)</f>
+        <f>_xlfn.XLOOKUP(B5,$H$5:$H$7,$I$5:$I$7)</f>
         <v/>
       </c>
       <c r="F5" s="10">
@@ -614,7 +614,7 @@
         <v>58.6</v>
       </c>
       <c r="E6" s="9">
-        <f>XLOOKUP(B6,$H$5:$H$7,$I$5:$I$7)</f>
+        <f>_xlfn.XLOOKUP(B6,$H$5:$H$7,$I$5:$I$7)</f>
         <v/>
       </c>
       <c r="F6" s="10">
@@ -648,7 +648,7 @@
         <v>37.9</v>
       </c>
       <c r="E7" s="9">
-        <f>XLOOKUP(B7,$H$5:$H$7,$I$5:$I$7)</f>
+        <f>_xlfn.XLOOKUP(B7,$H$5:$H$7,$I$5:$I$7)</f>
         <v/>
       </c>
       <c r="F7" s="10">
@@ -682,7 +682,7 @@
         <v>72.40000000000001</v>
       </c>
       <c r="E8" s="9">
-        <f>XLOOKUP(B8,$H$5:$H$7,$I$5:$I$7)</f>
+        <f>_xlfn.XLOOKUP(B8,$H$5:$H$7,$I$5:$I$7)</f>
         <v/>
       </c>
       <c r="F8" s="10">
@@ -708,7 +708,7 @@
         <v>61.3</v>
       </c>
       <c r="E9" s="9">
-        <f>XLOOKUP(B9,$H$5:$H$7,$I$5:$I$7)</f>
+        <f>_xlfn.XLOOKUP(B9,$H$5:$H$7,$I$5:$I$7)</f>
         <v/>
       </c>
       <c r="F9" s="10">
@@ -734,7 +734,7 @@
         <v>44.8</v>
       </c>
       <c r="E10" s="9">
-        <f>XLOOKUP(B10,$H$5:$H$7,$I$5:$I$7)</f>
+        <f>_xlfn.XLOOKUP(B10,$H$5:$H$7,$I$5:$I$7)</f>
         <v/>
       </c>
       <c r="F10" s="10">
@@ -760,7 +760,7 @@
         <v>68.09999999999999</v>
       </c>
       <c r="E11" s="9">
-        <f>XLOOKUP(B11,$H$5:$H$7,$I$5:$I$7)</f>
+        <f>_xlfn.XLOOKUP(B11,$H$5:$H$7,$I$5:$I$7)</f>
         <v/>
       </c>
       <c r="F11" s="10">
@@ -786,7 +786,7 @@
         <v>55.2</v>
       </c>
       <c r="E12" s="9">
-        <f>XLOOKUP(B12,$H$5:$H$7,$I$5:$I$7)</f>
+        <f>_xlfn.XLOOKUP(B12,$H$5:$H$7,$I$5:$I$7)</f>
         <v/>
       </c>
       <c r="F12" s="10">
@@ -809,7 +809,7 @@
         </is>
       </c>
       <c r="B15" s="6">
-        <f>XLOOKUP(B5,$H$5:$H$7,$I$5:$I$7)</f>
+        <f>_xlfn.XLOOKUP(B5,$H$5:$H$7,$I$5:$I$7)</f>
         <v/>
       </c>
       <c r="C15" s="10">
@@ -854,7 +854,7 @@
         </is>
       </c>
       <c r="B18" s="6">
-        <f>XLOOKUP("Lentils",$H$5:$H$7,$I$5:$I$7,"no price")</f>
+        <f>_xlfn.XLOOKUP("Lentils",$H$5:$H$7,$I$5:$I$7,"no price")</f>
         <v/>
       </c>
       <c r="C18" s="10">

</xml_diff>